<commit_message>
index: rebuild hero and footer after the Duna reference
Hero: full-bleed landscape in .hero-media with three masked blur layers and a
fade into the page background; copy anchored bottom-left. Nav is transparent at
the top of the page and gains its surface on scroll (.is-scrolled).

Footer: new shared src/components/Footer.astro used by MainLayout, LegalLayout
and BlogLayout. Single --ink block with divider, four link columns, legal row and
a landscape pinned to the bottom edge that dissolves into the background.

Placeholder JPEGs in public/images/ stand in until the final artwork is generated.
Design system: hero media and footer columns documented on /design-system/molecules,
--ink swatch added to atoms. PAGES.xlsx dates updated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAGES.xlsx
+++ b/PAGES.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pages" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Pages" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -540,12 +540,12 @@
       </c>
       <c r="H2" s="15" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="I2" s="15" t="inlineStr">
         <is>
-          <t>Main marketing landing page</t>
+          <t>Main marketing landing page. Redesign in progress on the redesign branch: full-bleed landscape hero, shared Footer component.</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
       </c>
       <c r="H3" s="15" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="I3" s="15" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="I4" s="15" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="H18" s="15" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="I18" s="15" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="H19" s="15" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="I19" s="15" t="inlineStr">
@@ -1386,12 +1386,12 @@
       </c>
       <c r="H20" s="15" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="I20" s="15" t="inlineStr">
         <is>
-          <t>Step, plan, testimonial, credibility, metric, case stat, case quote, speaker, form field, mobile menu link, author chip, author stack, post card, tag group, breadcrumb, author panel.</t>
+          <t>Step, plan, testimonial, credibility, metric, case stat, case quote, speaker, form field, mobile menu link, author chip, author stack, post card, tag group, breadcrumb, author panel. Hero media, footer columns.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
switcher: on / as well, and the collapse dot goes
The pill now ships on the live page with Live marked, so all five designs are
one click apart from wherever the reviewer lands. It is the only thing on
src/pages/index.astro that is not production, flagged in a comment there, in
CLAUDE.md and on the Home row of PAGES.xlsx, and it comes off before the page
ships.

The green dot that collapsed the pill is gone, and with it the toggle script
and the session-remembered state. Five links and a label need no chrome.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAGES.xlsx
+++ b/PAGES.xlsx
@@ -545,7 +545,7 @@
       </c>
       <c r="I2" s="15" t="inlineStr">
         <is>
-          <t>Main marketing landing page, the live design. The Duna-idiom redesign moved to /v1 on 2026-09-07; this page and global.css are production and are not touched by variation work.</t>
+          <t>Main marketing landing page, the live design. The Duna-idiom redesign moved to /v1 on 2026-09-07; this page and global.css are production and are not touched by variation work. Carries the temporary variation switcher (src/components/variants/VariantSwitcher.astro) for review on the redesign branch; remove it before shipping.</t>
         </is>
       </c>
     </row>
@@ -1758,7 +1758,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Design variations (/v1, /v1-1, /v2, /v3) are internal review routes: always Noindex, blocked in robots.txt, never in the sitemap. See CLAUDE.md, "Design variations".</t>
         </is>

</xml_diff>

<commit_message>
v1.1: forked from v1 as an exact copy
The page, the layout and the stylesheet are all copied: src/pages/v1-1/index.astro
on V11Layout, on src/styles/variants/v1-1.css. Nothing is shared with v1, so
/v1 stays exactly as the client saw it while v1.1 changes. Verified: adding a
rule to v1-1.css moves /v1-1 onto its own CSS asset and leaves /v1 untouched.
Identical stylesheets share one built asset because Vite hashes by content;
the sources are separate regardless.

variants.ts marks v1.1 ready, so the switcher stops dimming it.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAGES.xlsx
+++ b/PAGES.xlsx
@@ -1460,7 +1460,7 @@
       </c>
       <c r="D22" s="16" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Live</t>
         </is>
       </c>
       <c r="E22" s="17" t="inlineStr">
@@ -1470,7 +1470,7 @@
       </c>
       <c r="F22" s="15" t="inlineStr">
         <is>
-          <t>VariantStubLayout</t>
+          <t>V11Layout</t>
         </is>
       </c>
       <c r="G22" s="15" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="I22" s="15" t="inlineStr">
         <is>
-          <t>Placeholder for an iteration on v1. Not designed yet; the route exists so the variation switcher works.</t>
+          <t>Home page design variation v1.1, forked from v1 on 2026-09-07 as an exact copy and iterated from there. Own stylesheet src/styles/variants/v1-1.css and own layout V11Layout. noindex hard-coded in the layout, blocked in robots.txt, excluded from sitemap.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v2: the joindawn.com idiom on the client's copy
A dark opening with a split hero of two rounded cards, one circle whose arc
is drawn by scroll, a sunrise gradient into cream, then stacked sections with
rounded feet, a coverflow carousel for the audiences and a sky card for the
close. Source Serif 4 and Figtree, Dawn's orange, cream and ink palette,
gradient pills for every primary action. Own stylesheet (v2.css), own layout
(V2Layout) with Dawn's dark footer; the form and its scripts are v1's,
restyled. variants.ts marks v2 ready; PAGES.xlsx and CLAUDE.md updated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAGES.xlsx
+++ b/PAGES.xlsx
@@ -1507,7 +1507,7 @@
       </c>
       <c r="D23" s="16" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Live</t>
         </is>
       </c>
       <c r="E23" s="17" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="F23" s="15" t="inlineStr">
         <is>
-          <t>VariantStubLayout</t>
+          <t>V2Layout</t>
         </is>
       </c>
       <c r="G23" s="15" t="inlineStr">
@@ -1532,7 +1532,7 @@
       </c>
       <c r="I23" s="15" t="inlineStr">
         <is>
-          <t>Placeholder for a second design direction. Not designed yet.</t>
+          <t>Home page design variation v2, the joindawn.com idiom, built 2026-09-07. A dark cocoa ground the page opens on, a split hero of two rounded cards, one circle whose arc is drawn by scroll, a sunrise gradient into cream, then stacked sections with rounded feet, a coverflow carousel and a sky card. Source Serif 4 and Figtree. Own stylesheet src/styles/variants/v2.css and own layout V2Layout. noindex hard-coded in the layout, blocked in robots.txt, excluded from sitemap.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove the v1.1 design variation
The client dropped v1.1, so it goes out whole rather than sitting on the
switcher as a route nobody opens.

Deleted: src/pages/v1-1/index.astro, src/layouts/variants/V11Layout.astro,
src/styles/variants/v1-1.css, public/images/v1-1/ (both Bayshore renders)
and docs/v1-1-art-brief.md. The row is out of src/data/variants.ts, so the
switcher on / and on every remaining variation now lists Live, v1, v2 and
v3 only; out of the Disallow list in public/robots.txt, there being no
route left to block; and out of PAGES.xlsx. It was never in sitemap.xml.

CLAUDE.md and docs/v3-art-brief.md carry the same removal but are held
back from this commit: another session has uncommitted v3 work in both.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAGES.xlsx
+++ b/PAGES.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="32" customWidth="1" style="8" min="1" max="1"/>
@@ -1445,17 +1445,17 @@
     <row r="22" s="9">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>Design v1.1</t>
+          <t>Design v2</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>https://compoundhealth.io/v1-1</t>
+          <t>https://compoundhealth.io/v2</t>
         </is>
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>/v1-1</t>
+          <t>/v2</t>
         </is>
       </c>
       <c r="D22" s="16" t="inlineStr">
@@ -1470,12 +1470,12 @@
       </c>
       <c r="F22" s="15" t="inlineStr">
         <is>
-          <t>V11Layout</t>
+          <t>V2Layout</t>
         </is>
       </c>
       <c r="G22" s="15" t="inlineStr">
         <is>
-          <t>src/pages/v1-1/index.astro</t>
+          <t>src/pages/v2/index.astro</t>
         </is>
       </c>
       <c r="H22" s="15" t="inlineStr">
@@ -1485,24 +1485,24 @@
       </c>
       <c r="I22" s="15" t="inlineStr">
         <is>
-          <t>Home page design variation v1.1, forked from v1 on 2026-09-07. Answers the client feedback that v1 was not premium enough: bayshore.ai palette and gradient environments, square geometry, Cinzel Roman-caps labels, visible grid hairlines. Own stylesheet src/styles/variants/v1-1.css and own layout V11Layout. Both 3D renders are in, at public/images/v1-1/ (hero-monolith.webp, footer-stone.webp), see docs/v1-1-art-brief.md. noindex hard-coded in the layout, blocked in robots.txt, excluded from sitemap.</t>
+          <t>Home page design variation v2, the joindawn.com idiom, built 2026-09-07. A dark cocoa ground the page opens on, a split hero of two rounded cards, one circle whose arc is drawn by scroll, a sunrise gradient into cream, then stacked sections with rounded feet, a coverflow carousel and a sky card. Source Serif 4 and Figtree. Own stylesheet src/styles/variants/v2.css and own layout V2Layout. noindex hard-coded in the layout, blocked in robots.txt, excluded from sitemap.</t>
         </is>
       </c>
     </row>
     <row r="23" s="9">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>Design v2</t>
+          <t>Design v3</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
         <is>
-          <t>https://compoundhealth.io/v2</t>
+          <t>https://compoundhealth.io/v3</t>
         </is>
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
-          <t>/v2</t>
+          <t>/v3</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
@@ -1517,72 +1517,26 @@
       </c>
       <c r="F23" s="15" t="inlineStr">
         <is>
-          <t>V2Layout</t>
+          <t>V3Layout</t>
         </is>
       </c>
       <c r="G23" s="15" t="inlineStr">
         <is>
-          <t>src/pages/v2/index.astro</t>
+          <t>src/pages/v3/index.astro</t>
         </is>
       </c>
       <c r="H23" s="15" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="I23" s="15" t="inlineStr">
         <is>
-          <t>Home page design variation v2, the joindawn.com idiom, built 2026-09-07. A dark cocoa ground the page opens on, a split hero of two rounded cards, one circle whose arc is drawn by scroll, a sunrise gradient into cream, then stacked sections with rounded feet, a coverflow carousel and a sky card. Source Serif 4 and Figtree. Own stylesheet src/styles/variants/v2.css and own layout V2Layout. noindex hard-coded in the layout, blocked in robots.txt, excluded from sitemap.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" s="9">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>Design v3</t>
-        </is>
-      </c>
-      <c r="B24" s="15" t="inlineStr">
-        <is>
-          <t>https://compoundhealth.io/v3</t>
-        </is>
-      </c>
-      <c r="C24" s="15" t="inlineStr">
-        <is>
-          <t>/v3</t>
-        </is>
-      </c>
-      <c r="D24" s="16" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="E24" s="17" t="inlineStr">
-        <is>
-          <t>Noindex</t>
-        </is>
-      </c>
-      <c r="F24" s="15" t="inlineStr">
-        <is>
-          <t>V3Layout</t>
-        </is>
-      </c>
-      <c r="G24" s="15" t="inlineStr">
-        <is>
-          <t>src/pages/v3/index.astro</t>
-        </is>
-      </c>
-      <c r="H24" s="15" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="I24" s="15" t="inlineStr">
-        <is>
           <t>Home page design variation v3, the lassie.ai idiom, built 2026-09-10. One cream ground with no bands and no shadows, Newsreader at 350 standing in for ABC Marist plus DM Sans and DM Mono, a floating glass nav pill, and scroll used as a mechanism: the hero window closes on itself, three panels deal like a deck on a pinned stage, and six tiles orbit a scroll-scrubbed ellipse around a line that changes under them. Own stylesheet src/styles/variants/v3.css and own layout V3Layout. All four photographs are in at public/images/v3/; the hero and the closing frame were graded so white type reads without a scrim, per docs/v3-art-brief.md. noindex hard-coded in the layout, blocked in robots.txt, excluded from sitemap.</t>
         </is>
       </c>
     </row>
+    <row r="24" s="9"/>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="D2:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">

</xml_diff>

<commit_message>
v1: the Aeonik lockup, and the brand assets it needs
In-flight work from a concurrent session on this repo, committed here because
the whole tree was asked for. It brings Aeonik into public/fonts, a black
favicon, the v1 image set, and a BrandLockup and V1Logo pair, with the v1 page,
layout and stylesheet moved onto them. client_resources/ joins the ignore list
beside content_resources/, and PAGES.xlsx, variants.ts, V3Layout and the v3 art
brief carry the edits that came with it.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAGES.xlsx
+++ b/PAGES.xlsx
@@ -1433,12 +1433,12 @@
       </c>
       <c r="H21" s="15" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="I21" s="15" t="inlineStr">
         <is>
-          <t>Home page design variation v1, the Duna-idiom redesign moved off / on 2026-09-07. Own stylesheet src/styles/variants/v1.css. noindex hard-coded in the layout, blocked in robots.txt, excluded from sitemap.</t>
+          <t>Home page design variation v1, the client's final version, delivered 2026-09-11 as one flattened page and revised the same day (client_resources/compound-health-v1-new.html), applied to the project that day. The revision broke the curated note onto two lines above 640px, suppressed that break below it, and removed the hairline rule between the curated and partners sections. superpower.com's type scale and zinc / vermillion palette with the client's brand tones (rust, umber, bronze, moss) carrying the accent, Aeonik at 400 and 500, one white ground, a transparent nav that collapses into a blurred pill on scroll, a photographic hero card with the credibility items along its foot, auto-rotating discipline tabs, and a fixed footer the closing card uncovers. Photographs at public/images/v1/, faces at public/fonts/. Own lockup in V1Logo.astro; own stylesheet src/styles/variants/v1.css and own layout V1Layout. noindex hard-coded in the layout, blocked in robots.txt, excluded from sitemap.</t>
         </is>
       </c>
     </row>

</xml_diff>